<commit_message>
chore: save remaining storage engine adjustments
</commit_message>
<xml_diff>
--- a/sales_pipeline.xlsx
+++ b/sales_pipeline.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,6 +509,176 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Client (call_with_sarah.wav)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Pending Ai extraction</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Pending Ai extraction</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Client (call_with_john.mp3)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Pending Ai extraction</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Pending Ai extraction</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Harsha Johny</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>₹1200</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Send contract on friday</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Samantha Lee</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>₹5000</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Schedule demo for next week</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Rajesh Kumar</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>₹3000</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Follow up in 3 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Client (call_with_sarah.wav)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Pending Ai extraction</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Pending Ai extraction</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Client (call_with_john.mp3)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Pending Ai extraction</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Pending Ai extraction</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Harsha Johny</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>₹1200</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Send contract on friday</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Samantha Lee</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>₹5000</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Schedule demo for next week</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Rajesh Kumar</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>₹3000</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Follow up in 3 days</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: replace mock data loop with live gemini ai processing pipeline
</commit_message>
<xml_diff>
--- a/sales_pipeline.xlsx
+++ b/sales_pipeline.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,234 +448,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Test Company</t>
+          <t>Harsha from Kivali</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>$10,000</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Harsha Johny</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>₹1200</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Send contract on friday</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Samantha Lee</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>₹5000</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Schedule demo for next week</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Rajesh Kumar</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>₹3000</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Follow up in 3 days</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Client (call_with_sarah.wav)</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Pending Ai extraction</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Pending Ai extraction</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Client (call_with_john.mp3)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Pending Ai extraction</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Pending Ai extraction</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Harsha Johny</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>₹1200</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Send contract on friday</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Samantha Lee</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>₹5000</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Schedule demo for next week</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Rajesh Kumar</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>₹3000</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Follow up in 3 days</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Client (call_with_sarah.wav)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Pending Ai extraction</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Pending Ai extraction</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Client (call_with_john.mp3)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Pending Ai extraction</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Pending Ai extraction</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Harsha Johny</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>₹1200</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Send contract on friday</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Samantha Lee</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>₹5000</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Schedule demo for next week</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Rajesh Kumar</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>₹3000</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Follow up in 3 days</t>
+          <t>₹2,50,000</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Please send over the final service level agreement by this Friday for signing.</t>
         </is>
       </c>
     </row>

</xml_diff>